<commit_message>
docs: answer night-use question and clarify filter is not consumable
Row 20 now answers the second half of the question (studio/night-time
suitability) instead of giving the dB figure alone, with reference
points so 78dB is not read as quiet. Rows 6 and 16 state that the
magnetic filter is cleaned and reused rather than replaced, which was
missing from both and is a frequent customer question.

Supplier confirmed the 20-hour continuous-use figure and that Nellia
itself carries the warranty, so rows 19 and 4 stand as written.

Still open: paid-exchange price in row 21, and the wording of rows 9
and 13 on withdrawal limits, which is pending the owner's decision.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Nr3xSNVpjSWM8WArrddjYs
</commit_message>
<xml_diff>
--- a/docs/원룸만들기_상품상세정보_답변_S0000DUB.xlsx
+++ b/docs/원룸만들기_상품상세정보_답변_S0000DUB.xlsx
@@ -908,7 +908,8 @@
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t>무타공 벽걸이 마운트와 스타일링 노즐은 현재 별도판매 품목이 아닙니다.</t>
+          <t>무타공 벽걸이 마운트와 스타일링 노즐은 현재 별도판매 품목이 아닙니다.
+뒷면 마그네틱 필터는 교체형 소모품이 아닙니다. 자석식이라 손으로 떼어내 먼지를 털어 반복 사용하는 부품이며, 별도 판매하지 않습니다.</t>
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr">
@@ -1247,7 +1248,8 @@
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
-          <t>현재 고장으로 인한 A/S 외에 부속품을 교환은 불가능합니다.</t>
+          <t>현재 고장으로 인한 A/S 외에 부속품 교환은 불가능합니다.
+뒷면 마그네틱 필터는 교체형 소모품이 아니라 먼지를 털어 반복 사용하는 부품이라 교체 부품 목록에 포함되지 않습니다.</t>
         </is>
       </c>
       <c r="G17" s="8" t="inlineStr">
@@ -1375,7 +1377,9 @@
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>작동소음은 78dB입니다.</t>
+          <t>작동 소음은 78dB입니다. 드라이기 특성상 조용한 편은 아닙니다. (참고: 일반 대화가 약 60dB, 진공청소기가 70~80dB 수준입니다.)
+원룸이나 심야에 사용하실 때는 1단으로 쓰시면 풍속이 낮아지면서 소음도 함께 줄어듭니다.
+벽 거치 구조라 사용 후 서랍을 여닫을 일이 없어, 심야에는 그만큼 소리가 덜 납니다.</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr">

</xml_diff>

<commit_message>
docs: align withdrawal-limit wording with the Electronic Commerce Act
Rows 9 and 13 listed damaged packaging and a removed protective film as
grounds for refusing a return, but Article 17(2) expressly excludes
unpacking done to inspect the goods, and the packaging clause it does
contain is limited to copyable goods. Both are dropped, and row 13 now
states plainly that no depreciation schedule is operated — only the
statutory limits and the return shipping fee already set in row 10.

Rows 5 and 20 now record that 78dB is measured at speed 2.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Nr3xSNVpjSWM8WArrddjYs
</commit_message>
<xml_diff>
--- a/docs/원룸만들기_상품상세정보_답변_S0000DUB.xlsx
+++ b/docs/원룸만들기_상품상세정보_답변_S0000DUB.xlsx
@@ -877,7 +877,7 @@
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>78dB</t>
+          <t>78dB (2단 기준)</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
@@ -980,7 +980,7 @@
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>내용 확인을 위한 포장 개봉만으로 반품이 제한되지는 않습니다. 다만 포장 박스가 훼손되거나, 보호필름이 떨어진 경우와 고객 책임으로 제품이 훼손되거나 사용 및 일부 소비로 가치가 크게 감소한 경우에는 반품이 제한될 수 있습니다.</t>
+          <t>내용 확인을 위한 포장 개봉만으로 반품이 제한되지는 않습니다. 다만 고객 책임으로 제품이 훼손되거나 사용 및 일부 소비로 가치가 크게 감소한 경우에는 반품이 제한될 수 있습니다.</t>
         </is>
       </c>
       <c r="G9" s="8" t="inlineStr">
@@ -1147,7 +1147,10 @@
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>포장 개봉만으로 감가하지 않습니다. 고객 책임으로 상품 가치가 실제로 감소한 경우에만 사전 고지된 기준을 적용할 수 있으며, 포장재 훼손 및 구성품 파손 등은 감가 공제가 아니라 전체 금액을 부담하여야 합니다. 재판매가 어렵습니다.</t>
+          <t>포장을 열어 내용을 확인한 것만으로는 감가하거나 반품을 제한하지 않습니다.
+반품이 제한되는 경우는 소비자 책임으로 제품이 멸실·훼손되었거나, 사용 또는 일부 소비로 제품 가치가 현저히 감소한 경우입니다. 이에 해당하는지는 넬리아가 사진 등으로 확인한 뒤 고객께 안내드립니다.
+포장재의 통상적인 개봉 흔적은 반품 제한 사유나 감가 사유로 적용하지 않습니다.
+별도의 감가 공제율은 운영하지 않으며, 단순 변심 반품의 경우 반송비(편도 3,000원 / 왕복 6,000원, 도서산간 5,000원 추가)만 고객이 부담합니다.</t>
         </is>
       </c>
       <c r="G14" s="8" t="inlineStr">
@@ -1377,7 +1380,7 @@
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>작동 소음은 78dB입니다. 드라이기 특성상 조용한 편은 아닙니다. (참고: 일반 대화가 약 60dB, 진공청소기가 70~80dB 수준입니다.)
+          <t>작동 소음은 2단(최대) 기준 78dB입니다. 드라이기 특성상 조용한 편은 아닙니다. (참고: 일반 대화가 약 60dB, 진공청소기가 70~80dB 수준입니다.)
 원룸이나 심야에 사용하실 때는 1단으로 쓰시면 풍속이 낮아지면서 소음도 함께 줄어듭니다.
 벽 거치 구조라 사용 후 서랍을 여닫을 일이 없어, 심야에는 그만큼 소리가 덜 납니다.</t>
         </is>

</xml_diff>